<commit_message>
Reset adult Posted flags for fresh start on new channel
The 3 previously-posted riddles only went to the now-disabled
channel, so clear their Posted? + stale links to re-publish fresh.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Riddle_Content_Bank.xlsx
+++ b/Riddle_Content_Bank.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me &amp; Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Adult Riddles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Kids Riddles" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Adult – Original" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kids – Original" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me &amp; Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adult Riddles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kids Riddles" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adult – Original" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kids – Original" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Adult Riddles'!$A$1:$I$1</definedName>
@@ -9628,14 +9628,10 @@
       </c>
       <c r="F2" s="55" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G2" s="57" t="inlineStr">
-        <is>
-          <t>https://youtu.be/nHgUWCiPPU8</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G2" s="57" t="n"/>
     </row>
     <row r="3" ht="31.5" customHeight="1" s="32">
       <c r="A3" s="58" t="n">
@@ -9663,14 +9659,10 @@
       </c>
       <c r="F3" s="58" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G3" s="60" t="inlineStr">
-        <is>
-          <t>https://youtu.be/piWoV4Zx9wY</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" s="60" t="n"/>
     </row>
     <row r="4" ht="31.5" customHeight="1" s="32">
       <c r="A4" s="55" t="n">
@@ -9698,14 +9690,10 @@
       </c>
       <c r="F4" s="55" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G4" s="57" t="inlineStr">
-        <is>
-          <t>https://youtu.be/maDijb1uzF8</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" s="57" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="32">
       <c r="A5" s="58" t="n">
@@ -10234,6 +10222,7 @@
       </c>
       <c r="G21" s="60" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="32">
       <c r="A23" s="61" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
content: add 100 riddles (No.201-300) + raise Adult Riddles read bound to 301
</commit_message>
<xml_diff>
--- a/Riddle_Content_Bank.xlsx
+++ b/Riddle_Content_Bank.xlsx
@@ -1087,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:I301"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="31" min="1" max="1"/>
@@ -9744,6 +9744,3806 @@
       <c r="I201" s="55" t="inlineStr">
         <is>
           <t>https://youtu.be/WriLkPPlosM</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="n">
+        <v>29</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>I have teeth of metal but never chew; drag me through cheese and I'll shred it for you. What am I?</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>A grater</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="n">
+        <v>29</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Twist me down and I'll bite the cork, then pull it free without a fork. What am I?</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>A corkscrew</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="n">
+        <v>29</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>I roll back and forth but go nowhere at all, flattening dough till it's thin on the wall. What am I?</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>A rolling pin</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="n">
+        <v>30</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>I catch every drip and hold every soak, then wring myself dry at a squeeze or a choke. What am I?</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>A dishcloth</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="n">
+        <v>30</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>I keep your leftovers cold through the night, humming in darkness behind a shut light. What am I?</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>A refrigerator</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="n">
+        <v>30</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Spin my plate and I'll warm your meal, in seconds of hum you can hear but not feel. What am I?</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>A microwave</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="n">
+        <v>30</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>I press out your wrinkles with heat and with steam, then stand up on end when I've finished the seam. What am I?</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>An iron</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="n">
+        <v>30</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>I swallow the dust from under your feet, dragged room to room on a cord you repeat. What am I?</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>A vacuum</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="n">
+        <v>30</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>I mop up the floor from a bucket of grey, then hang up to dry at the end of the day. What am I?</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>A mop</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" t="n">
+        <v>30</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>I hug just one toe-to-heel each day, worn out in pairs then thrown away. What am I?</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>A sock</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" t="n">
+        <v>31</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>I circle your waist and I hold up your pants, tightened a notch after too many chances. What am I?</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>A belt</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="n">
+        <v>31</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>I ride on your back but I carry no weight of my own, filled up with books till your shoulders have grown. What am I?</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>A backpack</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="n">
+        <v>31</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>I hammer no nail yet I answer to swings; grip me to loosen the tightest of things. What am I?</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>A wrench</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="n">
+        <v>31</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>I turn and I turn but I travel nowhere, biting the wood till I'm buried in there. What am I?</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>A screw</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="n">
+        <v>31</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>I let a door swing and I let a lid lift; I fold in the middle, my one only gift. What am I?</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>A hinge</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" t="n">
+        <v>31</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>I coil up tight then I leap when set free, storing your push till you finally see. What am I?</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>A spring</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" t="n">
+        <v>31</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Six strings on my neck and a hole in my chest; strum me for songs at a campfire's request. What am I?</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>A guitar</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" t="n">
+        <v>32</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>I keep the beat with a tick and a sway, never a note but I show you the way. What am I?</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>A metronome</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" t="n">
+        <v>32</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>I spin round and round with a needle on top, and music pours out till you lift it to stop. What am I?</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>A record</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" t="n">
+        <v>32</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>I fall in the autumn, I'm green in the spring; I feed the whole tree yet I'm such a thin thing. What am I?</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>A leaf</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" t="n">
+        <v>32</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Buried in darkness, I wait for the rain, then split myself open to start it again. What am I?</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>A seed</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" t="n">
+        <v>32</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>I hoard my own water in a coat full of spears, standing in deserts for hundreds of years. What am I?</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>A cactus</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" t="n">
+        <v>32</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>I'm a mountain of water that falls off a cliff, roaring so loud you can feel the earth shift. What am I?</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>A waterfall</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" t="n">
+        <v>32</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Most of me hides where the cold currents flow; ships fear the tenth of me that doesn't show. What am I?</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>An iceberg</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" t="n">
+        <v>33</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>I hang from the gutter and grow with the cold, a dagger of water the winter has told. What am I?</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>An icicle</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" t="n">
+        <v>33</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>I'm a river of ice that crawls down the hill, carving the valley then leaving it still. What am I?</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>A glacier</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" t="n">
+        <v>33</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Closed I am woody, a fist full of seed; open in warmth I let the wind lead. What am I?</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>A pinecone</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" t="n">
+        <v>33</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>You bring me up close to bring far things near; the stars fill my eye when the night sky is clear. What am I?</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>A telescope</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" t="n">
+        <v>33</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>I make the invisible leap into view, blowing up specks that were too small for you. What am I?</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>A microscope</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" t="n">
+        <v>33</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>I split the white light into ribbons of hue, a triangle prism of red into blue. What am I?</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>A prism</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" t="n">
+        <v>33</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>I blast off with fire and I climb past the sky, shedding my stages the higher I fly. What am I?</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>A rocket</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" t="n">
+        <v>34</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>I circle the earth without touching the ground, bouncing your signals back safe and sound. What am I?</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>A satellite</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" t="n">
+        <v>34</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>I trail a bright tail as I swing past the sun, then vanish for lifetimes when my visit is done. What am I?</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>A comet</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" t="n">
+        <v>34</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>I dive without gills and I sail without wind, hiding in silence with sonar to find. What am I?</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>A submarine</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" t="n">
+        <v>34</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>I lift you in floors without climbing a stair, a box on a cable that carries you there. What am I?</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>An elevator</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" t="n">
+        <v>34</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>I bloom in the wind on a string you hold tight, tugging to climb to a paper-thin height. What am I?</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>A kite</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" t="n">
+        <v>34</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>I catch all the wind so a boat can move on; without me the sailor's swift journey is gone. What am I?</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>A sail</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" t="n">
+        <v>34</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Red, amber, green — I command every street, and cars hold their breath till my green says proceed. What am I?</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>A traffic light</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" t="n">
+        <v>35</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>I mark where you'll type with a blink and a bar, waiting on screen wherever you are. What am I?</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>A cursor</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" t="n">
+        <v>35</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Put a pound in my front and a topic behind, and suddenly thousands of posts you can find. What am I?</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>A hashtag</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" t="n">
+        <v>35</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>I'm the tiniest square that a screen can display; a million of me make the picture okay. What am I?</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>A pixel</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" t="n">
+        <v>35</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>I guard your machine from the traffic outside, deciding what enters and what is denied. What am I?</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>A firewall</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" t="n">
+        <v>35</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>A site drops me quietly to help it recall who you are on return, though I'm not sweet at all. What am I?</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>A cookie</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" t="n">
+        <v>35</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Blue and underlined, I whisk you away; one click and a whole other page is in play. What am I?</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>A hyperlink</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" t="n">
+        <v>35</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>I read a striped forehead of black and of white, and beep out a price at the checkout tonight. What am I?</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>A barcode</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" t="n">
+        <v>36</v>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>A camera that watches wherever you roam online, I show your own face on a call that's on time. What am I?</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>A webcam</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" t="n">
+        <v>36</v>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>I sit in a bowl of my own quiet steam, then poured into cups I'm the color of dream. Bag me or leaf me, I turn water to brew. What am I?</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Tea</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" t="n">
+        <v>36</v>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>I circle your wrist and I count out your run, buzzing your steps till the walking is done. What am I?</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>A fitness tracker</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" t="n">
+        <v>36</v>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>I remember your logins, your cards, and your keys, locked in one vault that you open with ease. What am I?</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>A password manager</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" t="n">
+        <v>36</v>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>I keep a whole book in a slab you can hold, thousands of pages but nothing to fold. What am I?</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>An e-reader</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" t="n">
+        <v>36</v>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>I stand at the door with an eye and a chime, showing your porch on your phone anytime. What am I?</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>A doorbell camera</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" t="n">
+        <v>36</v>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>You speak and I listen from cross the whole room, dimming the lights or predicting the gloom. What am I?</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>A smart speaker</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" t="n">
+        <v>37</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>I am not a lie, but I'm not quite the truth; a story you tell to a gullible youth. Half-real, I grow with each telling anew. What am I?</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>An exaggeration</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" t="n">
+        <v>37</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>I count myself down till I hit at zero, then buzz or explode as the clock's little hero. What am I?</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>A countdown</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" t="n">
+        <v>37</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>I am the line where the sea meets the sky, always ahead, though you'll never draw nigh. What am I?</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>The horizon</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" t="n">
+        <v>37</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>I'm the promise of doing before it's too late; miss me and everyone circles the date. What am I?</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>A deadline</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" t="n">
+        <v>37</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>I am dropped in a box or I'm tapped on a screen; count all of me up and I crown a new queen or king. What am I?</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>A vote</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="n">
+        <v>37</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>I repeat what you did without asking you twice, hard to break loose and not always nice. What am I?</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>A habit</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" t="n">
+        <v>37</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>I prove you were elsewhere when trouble occurred, a story with witnesses, checked word for word. What am I?</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>An alibi</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" t="n">
+        <v>38</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>I'm the space you leave blank between word and word, without me a sentence would sound quite absurd. What am I?</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>A space</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="n">
+        <v>38</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>The more of me you take, the more you leave behind; I follow you walking but I'm not far behind. What am I?</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>A footstep</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="n">
+        <v>38</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>I have hands but no fingers, a face but no eyes; I run all day long but I stay the same size. What am I?</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>A clock</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" t="n">
+        <v>38</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>I chime on the hour with a swing and a weight, a grandfather standing that's never once late. What am I?</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>A pendulum clock</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" t="n">
+        <v>38</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>I have keys but no locks, space but no room; you enter me daily but I'm not a tomb. What am I?</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>A keyboard</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" t="n">
+        <v>38</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>I'm gold in the morning and cold in the night; I feed the whole world but I'm blinding to sight. What am I?</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>The sun</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" t="n">
+        <v>38</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>I wax and I wane and I borrow my light; I pull at the tides every single night. What am I?</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>The moon</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" t="n">
+        <v>39</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>I fall without hurting, I break without sound; I paint the whole town without touching the ground. What am I?</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Snow</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" t="n">
+        <v>39</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>You throw away my outside and cook my inside, then eat my outside and throw my inside. What am I?</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Corn on the cob</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" t="n">
+        <v>39</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>I have a ring for each year that I've grown, counted in circles once I've been thrown. What am I?</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>A tree trunk</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="n">
+        <v>39</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>I'm light as a feather, yet the strongest can't hold me for much more than a minute or so. What am I?</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>A breath</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="n">
+        <v>39</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Feed me and I grow tall and bright; give me a drink and I die in the night. What am I?</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>A fire</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="n">
+        <v>39</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>I'm the fifth if you letter my days of the week; find me in 'time' but in 'clock' I don't speak. What am I?</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>The letter T</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Wordplay</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="n">
+        <v>39</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>I'm easy to get into but hard to get out; the deeper you're in me, the more you'll dig about. What am I?</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Trouble</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="n">
+        <v>40</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Forwards I'm heavy, but backwards I'm not; read me both ways for the trick that I've got. What am I?</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>The word 'ton'</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Wordplay</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="n">
+        <v>40</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Give me food and I live; give me water and I die. Orange and flickering, I dance in the sky. What am I?</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>A flame</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="n">
+        <v>40</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>I ring without a mouth and run without a leg; a chime in your pocket you answer or beg. What am I?</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>A phone</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" t="n">
+        <v>40</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>I sit between two players and settle each fight, awarding the point with a whistle so bright. What am I?</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>A referee</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="n">
+        <v>40</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>I have a neck and a body but no arms at all; fill me with flowers to stand tall and proud. What am I?</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>A vase</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="n">
+        <v>40</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>I carry your voice to a friend far away, folded and stamped for the mail-carrier's tray. What am I?</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>A letter</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="n">
+        <v>40</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>I keep perfect time without gears or a spring; I follow the sun as it circles to bring my shadow around like a slow-moving thing. What am I?</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>A sundial</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="n">
+        <v>41</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>I flip your pancakes with a slide and a lift, wide and flat is my one only gift. What am I?</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>A spatula</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="n">
+        <v>41</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>I scoop out the soup with a deep little bowl on a long metal arm. What am I?</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>A ladle</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="n">
+        <v>41</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>I sense the room's warmth and I argue with it, turning the heat up or down bit by bit. What am I?</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>A thermostat</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="n">
+        <v>41</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>A doctor puts me in her ears to hear the drum of a beating so near. What am I?</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>A stethoscope</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="n">
+        <v>41</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>I bite once with a needle so thin, pushing the medicine under your skin. What am I?</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>A syringe</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" t="n">
+        <v>41</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>I wrap up a cut and I soak up the sore, sticking to skin till you need me no more. What am I?</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>A bandage</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" t="n">
+        <v>41</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>I lend you a leg when your own one is broken, tucked under your arm as a healing token. What am I?</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>A crutch</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" t="n">
+        <v>42</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Four wheels and a plank, I roll under your feet; kick once and I carry you down the whole street. What am I?</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>A skateboard</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="n">
+        <v>42</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>I'm a staircase that moves so your feet needn't climb; step on and I carry you up every time. What am I?</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>An escalator</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="n">
+        <v>42</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>I spin one at a time to let the crowd through, counting each body that passes on cue. What am I?</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>A turnstile</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="n">
+        <v>42</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>I bend like a horn but I sing like a reed; press down my keys for the jazz that you need. What am I?</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>A saxophone</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="n">
+        <v>42</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Cup me in your hands and breathe in and out; I hum out a blues with a bend and a shout. What am I?</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>A harmonica</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="n">
+        <v>42</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Strike my wooden bars with a mallet or two, and a ladder of notes comes ringing to you. What am I?</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>A xylophone</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="n">
+        <v>42</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Shake me or slap me, I jingle and ring, a circle of bells is the music I bring. What am I?</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>A tambourine</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="n">
+        <v>43</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Three valves and a bell, I blare loud and bright; press me for fanfares that carry for miles. What am I?</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>A trumpet</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" t="n">
+        <v>43</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Yellow when young, then I turn my head grey; blow on my seeds and they scatter away. What am I?</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>A dandelion</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" t="n">
+        <v>43</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Hold me to your ear on the sand by the sea, and the sound of the ocean is captured in me. What am I?</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>A seashell</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" t="n">
+        <v>43</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>I spin the water down into a swallowing throat, dragging under whatever won't stay afloat. What am I?</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>A whirlpool</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" t="n">
+        <v>43</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>I burst from the ground in a fountain of steam, boiling and timed like the earth's own dream. What am I?</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>A geyser</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" t="n">
+        <v>43</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>I twist from the sky in a funnel of wind, flinging up houses wherever I've been. What am I?</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>A tornado</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>